<commit_message>
mapa przeplywu z macierz_CX.xlsx: zakladka Przeplyw (Z, Do, Etykieta, Scenariusz, Opcjonalny), skrypt add-flow-sheet.py, adapter cj-flow-adapter.js, filtr scenariusza i przelacznik Real/Demo
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/macierz_CX_demo.xlsx
+++ b/macierz_CX_demo.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Mapowanie_PP_RC" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Mapowanie_RC_IN" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Dane" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Przepływ" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Macierz CX'!$A$1:$Z$61</definedName>
@@ -9922,4 +9923,849 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Z (Touchpoint ID)</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>Do (Touchpoint ID)</t>
+        </is>
+      </c>
+      <c r="C1" s="13" t="inlineStr">
+        <is>
+          <t>Etykieta</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
+          <t>Scenariusz</t>
+        </is>
+      </c>
+      <c r="E1" s="13" t="inlineStr">
+        <is>
+          <t>Opcjonalny (tak/nie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TP047</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TP036</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TP036</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TP037</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TP037</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TP048</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TP048</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TP003</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TP003</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TP038</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TP038</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TP049</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TP049</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TP051</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TP051</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TP004</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TP004</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TP039</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TP039</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TP005</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TP005</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TP050</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TP050</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TP006</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TP006</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TP007</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TP007</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TP061</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TP061</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TP062</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TP062</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>TP008</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TP008</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TP009</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TP009</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>TP010</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TP010</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>TP011</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TP011</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>TP012</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TP012</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TP040</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TP040</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>TP013</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>TP013</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>TP014</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>TP014</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>TP015</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TP015</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>TP052</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TP052</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>TP053</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TP053</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>TP016</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TP016</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>TP017</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>TP017</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>TP018</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>TP018</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>TP054</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>TP054</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>TP019</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>TP019</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>TP020</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>TP020</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>TP021</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>TP021</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>TP022</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>TP022</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>TP023</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>TP023</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>TP024</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>TP024</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>TP025</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>TP025</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>TP026</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>TP026</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>TP027</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>TP027</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TP041</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>TP041</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TP028</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>TP028</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>TP042</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>TP042</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>TP043</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>TP043</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>TP055</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>TP055</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>TP029</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>TP029</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>TP030</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>TP030</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>TP031</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>TP031</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>TP032</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>TP032</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>TP044</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>TP044</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>TP056</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>TP056</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>TP033</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>TP033</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>TP034</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>TP034</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>TP045</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>TP045</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>TP057</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>TP057</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>TP058</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>TP058</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>TP059</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>TP059</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>TP035</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>TP035</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>TP046</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>TP046</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>TP060</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>TP038</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>TP048</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>powrót po braku odpowiedzi (DEMO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>TP004</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>TP049</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>ponowne zapytanie (DEMO)</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Serwis</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>TP037</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>TP049</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>skrót (DEMO)</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>TP005</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>TP006</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>alternatywa (DEMO)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Serwis</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Nieznany punkt" error="Wybierz Touchpoint ID z zakładki Macierz CX." sqref="A2:B500">
+      <formula1>'Macierz CX'!$D$2:$D$500</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E500">
+      <formula1>"tak,nie"</formula1>
+    </dataValidation>
+  </dataValidations>
+</worksheet>
 </file>
</xml_diff>